<commit_message>
Temporarily set Phase 2 duration to 30 seconds for testing
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F4A98D-EA01-4EB0-A9C9-5E329EDEAE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506A0F81-661F-4C7E-A46C-69A40693561D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1515" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>19.40</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>320851d</t>
+  </si>
+  <si>
+    <t>66aae37</t>
+  </si>
+  <si>
+    <t>17.33</t>
+  </si>
+  <si>
+    <t>AutoFokus funktioniert auf IOS, Face1Recall werden Bilder noch nicht korrekt geladen.</t>
   </si>
 </sst>
 </file>
@@ -447,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:D10"/>
+  <dimension ref="B7:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -455,7 +464,7 @@
     <col min="4" max="4" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>46075</v>
       </c>
@@ -466,7 +475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>46079</v>
       </c>
@@ -477,7 +486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>46079</v>
       </c>
@@ -488,7 +497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>46079</v>
       </c>
@@ -497,6 +506,20 @@
       </c>
       <c r="D10" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="3">
+        <v>46083</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Face2Task with MathTask integration and restore production phase timers
- Add MathTask integration to Face2Task with memory distraction between rounds
- Implement multi-round system: Level 1 (4 rounds), Level 2 (5 rounds), Level 3 (6 rounds)
- Add face position shuffling after each MathTask completion
- Prevent duplicate face selections across rounds within single task
- Fix point awarding system: MathTask points immediate, Face2Task points at end
- Add double-click protection and processing locks
- Restore phase timers to production values: Phase 1 (180s), Phase 2 (180s), Phase 3 (240s)
- Ensure MathTask points display immediately in ScoreDisplay
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506A0F81-661F-4C7E-A46C-69A40693561D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90641E65-8A01-4D6B-B17C-FAAE143AAE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
+    <workbookView xWindow="2730" yWindow="1560" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>19.40</t>
   </si>
@@ -69,6 +69,15 @@
   </si>
   <si>
     <t>AutoFokus funktioniert auf IOS, Face1Recall werden Bilder noch nicht korrekt geladen.</t>
+  </si>
+  <si>
+    <t>07.52</t>
+  </si>
+  <si>
+    <t>595e7bc</t>
+  </si>
+  <si>
+    <t>Face1 Recall Bilder werden korrekt geladen, MathTask in Face2Task noch nicht integriert. Phase 1 und 2 jeweils 30 sec.</t>
   </si>
 </sst>
 </file>
@@ -456,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:F11"/>
+  <dimension ref="B7:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -522,6 +531,20 @@
         <v>10</v>
       </c>
     </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="3">
+        <v>46084</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
MathTask Integration und JSX Fixes - MathTask in alle Task-Komponenten integriert (Chess, Hand, Face1, Face2, Pie) - JSX Syntax-Fehler behoben - Overlay-Scrolling verhindert - Punkte-Animation entfernt
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90641E65-8A01-4D6B-B17C-FAAE143AAE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03DAD95-A41B-4234-BE80-A35D9AF2D2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="1560" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
+    <workbookView xWindow="2730" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>19.40</t>
   </si>
@@ -78,13 +78,25 @@
   </si>
   <si>
     <t>Face1 Recall Bilder werden korrekt geladen, MathTask in Face2Task noch nicht integriert. Phase 1 und 2 jeweils 30 sec.</t>
+  </si>
+  <si>
+    <t>6e6c961</t>
+  </si>
+  <si>
+    <t>12.15</t>
+  </si>
+  <si>
+    <t>10.38</t>
+  </si>
+  <si>
+    <t>3bb4734</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,6 +115,11 @@
       <sz val="14"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -125,12 +142,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -465,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:F12"/>
+  <dimension ref="B7:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -545,6 +563,28 @@
         <v>13</v>
       </c>
     </row>
+    <row r="13" spans="2:6" ht="20.25" x14ac:dyDescent="0.35">
+      <c r="B13" s="3">
+        <v>46084</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="3">
+        <v>46094</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Face components loading & implement universal image preloading
- Fixed Face1Recall, Face2Recall, Face2Task loading issues by removing legacy loading states
- Implemented universal image preloading strategy (all 91 images at startup)
- Added MobileErrorBoundary component for Android crash prevention
- Added mobile optimization utilities with HMR stability improvements
- Fixed iOS detection logic and mobile compatibility
- Reduced Phase 2 timer from 180s to 30s for testing
- Updated OptimizedImage component for better mobile support
- Removed complex device-specific loading in favor of simple universal approach
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03DAD95-A41B-4234-BE80-A35D9AF2D2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C46FFEF-302C-40F1-B261-53A00126C584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>19.40</t>
   </si>
@@ -90,13 +90,49 @@
   </si>
   <si>
     <t>3bb4734</t>
+  </si>
+  <si>
+    <t>10.13</t>
+  </si>
+  <si>
+    <t>546f10e</t>
+  </si>
+  <si>
+    <t>Punkte Felder entfernt railway service name geändert distractor-web</t>
+  </si>
+  <si>
+    <t>f2d7271</t>
+  </si>
+  <si>
+    <t>15.15</t>
+  </si>
+  <si>
+    <t>MathTask Zahl angeglichen. TaskExamples scrollbar</t>
+  </si>
+  <si>
+    <t>11.58</t>
+  </si>
+  <si>
+    <t>4c0353b</t>
+  </si>
+  <si>
+    <t>Web Socket Fehler korrigiert</t>
+  </si>
+  <si>
+    <t>8193c2f</t>
+  </si>
+  <si>
+    <t>14.17</t>
+  </si>
+  <si>
+    <t>Bildladevorgang für neuere &gt;IOS Versionen aktualisiert</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +157,11 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -142,13 +183,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -483,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:F14"/>
+  <dimension ref="B7:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -585,7 +630,64 @@
         <v>17</v>
       </c>
     </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="3">
+        <v>46098</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="3">
+        <v>46098</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="3">
+        <v>46106</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="3">
+        <v>46106</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Face1Task iOS loading + Add iOS debugging logs
- Fixed Face1Task: Removed isReady loading delay blocking images on iOS
- Added extensive iOS debugging logs in OptimizedImage to diagnose iPhone issues
- Debug logs will show iOS detection, userAgent, loading attempts, and errors
- This will help identify why Face1Task images don't load on newest iOS devices
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C46FFEF-302C-40F1-B261-53A00126C584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB63C38-9EAD-4180-967A-1F264639337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>19.40</t>
   </si>
@@ -126,6 +126,15 @@
   </si>
   <si>
     <t>Bildladevorgang für neuere &gt;IOS Versionen aktualisiert</t>
+  </si>
+  <si>
+    <t>10.15</t>
+  </si>
+  <si>
+    <t>6fc20bd</t>
+  </si>
+  <si>
+    <t>Phase 1 und Phase 2 verkürzt, Bilder werden alle am Anfang geladen.</t>
   </si>
 </sst>
 </file>
@@ -528,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:F18"/>
+  <dimension ref="B7:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -686,6 +695,20 @@
         <v>29</v>
       </c>
     </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="3">
+        <v>46110</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Update to version 2026v002 - synchronized version numbers across all language files
</commit_message>
<xml_diff>
--- a/GIT Version.xlsx
+++ b/GIT Version.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\areim\Documents\WEBAPPS\distractor-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB63C38-9EAD-4180-967A-1F264639337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58CBC7B-C937-40CC-9B1E-CD127E02B715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="840" windowWidth="21735" windowHeight="14640" xr2:uid="{52E9E515-A856-4913-8076-17DA4FA96A63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>19.40</t>
   </si>
@@ -135,6 +135,15 @@
   </si>
   <si>
     <t>Phase 1 und Phase 2 verkürzt, Bilder werden alle am Anfang geladen.</t>
+  </si>
+  <si>
+    <t>eb27e47</t>
+  </si>
+  <si>
+    <t>10.32</t>
+  </si>
+  <si>
+    <t>IOS Bilder funktionieren auf allen Versionen, Phase 1 und 2 noch 30 Sekunden</t>
   </si>
 </sst>
 </file>
@@ -537,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BEAAB03-D1B3-4B4E-99FF-44A3536525FE}">
-  <dimension ref="B7:F19"/>
+  <dimension ref="B7:F20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -709,6 +718,20 @@
         <v>32</v>
       </c>
     </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="3">
+        <v>46121</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>